<commit_message>
Add cover and back image URLs, and store names as family, given.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/master our program.xlsx
+++ b/master our program.xlsx
@@ -33,7 +33,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,12 +64,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -432,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1"/>
+  <dimension ref="A1:AR1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" customWidth="1" min="1" max="1"/>
@@ -477,6 +485,8 @@
     <col width="13" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="28" customWidth="1" min="43" max="43"/>
+    <col width="28" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
@@ -688,6 +698,16 @@
       <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Config 1</t>
+        </is>
+      </c>
+      <c r="AQ1" s="3" t="inlineStr">
+        <is>
+          <t>Cover image URL</t>
+        </is>
+      </c>
+      <c r="AR1" s="3" t="inlineStr">
+        <is>
+          <t>Back image URL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add named scan lists, scanner IDs with approve/final, and checkbox filters to keep or clear books.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/master our program.xlsx
+++ b/master our program.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR1"/>
+  <dimension ref="A1:AS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,7 @@
     <col width="13" customWidth="1" min="42" max="42"/>
     <col width="28" customWidth="1" min="43" max="43"/>
     <col width="28" customWidth="1" min="44" max="44"/>
+    <col width="22" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
@@ -708,6 +709,11 @@
       <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>Back image URL</t>
+        </is>
+      </c>
+      <c r="AS1" s="3" t="inlineStr">
+        <is>
+          <t>Scanner ID</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add orange Translator, Illustrator, MARC, and DDC columns.
Collect these fields when bookstore or National Library pages expose them, and restore tight spacing in the book list.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/master our program.xlsx
+++ b/master our program.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,10 @@
     <col width="28" customWidth="1" min="43" max="43"/>
     <col width="28" customWidth="1" min="44" max="44"/>
     <col width="22" customWidth="1" min="45" max="45"/>
+    <col width="22" customWidth="1" min="46" max="46"/>
+    <col width="22" customWidth="1" min="47" max="47"/>
+    <col width="22" customWidth="1" min="48" max="48"/>
+    <col width="22" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
@@ -714,6 +718,26 @@
       <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>Scanner ID</t>
+        </is>
+      </c>
+      <c r="AT1" s="3" t="inlineStr">
+        <is>
+          <t>Translator</t>
+        </is>
+      </c>
+      <c r="AU1" s="3" t="inlineStr">
+        <is>
+          <t>Illustrator</t>
+        </is>
+      </c>
+      <c r="AV1" s="3" t="inlineStr">
+        <is>
+          <t>MARC</t>
+        </is>
+      </c>
+      <c r="AW1" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
         </is>
       </c>
     </row>

</xml_diff>